<commit_message>
Inclusão script de remoção BR3
</commit_message>
<xml_diff>
--- a/Planilhas/Pedidos - CC.xlsx
+++ b/Planilhas/Pedidos - CC.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\python_scripts\Planilhas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\python_scripts\PLANILHAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF3D87DB-ED18-4B8A-A31D-557DE83B694D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F17A6421-4AE8-41D9-A3C6-0C95F2FBEB6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" xr2:uid="{B22F4247-8A78-4CA2-917D-234C68224E18}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="6">
   <si>
     <t>Item</t>
   </si>
@@ -193,8 +193,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C4F11308-4C43-48B9-BA07-AEB362118F73}" name="Tabela1" displayName="Tabela1" ref="A1:E183" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
-  <autoFilter ref="A1:E183" xr:uid="{C4F11308-4C43-48B9-BA07-AEB362118F73}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C4F11308-4C43-48B9-BA07-AEB362118F73}" name="Tabela1" displayName="Tabela1" ref="A1:E202" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
+  <autoFilter ref="A1:E202" xr:uid="{C4F11308-4C43-48B9-BA07-AEB362118F73}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{D0BC8C79-FDF1-4144-B598-1BCD4BB7CFD1}" name="Pedidos"/>
     <tableColumn id="2" xr3:uid="{3D9316E3-CFBE-4A9E-8B75-E0BF8E30E135}" name="Item" dataDxfId="3"/>
@@ -503,7 +503,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C176DAE8-01D4-4562-9DC5-3FF54C0846F5}">
-  <dimension ref="A1:E183"/>
+  <dimension ref="A1:E202"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.81640625" bestFit="1" customWidth="1"/>
@@ -532,7 +532,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2">
-        <v>4500034383</v>
+        <v>4500037725</v>
       </c>
       <c r="B2">
         <v>10</v>
@@ -543,7 +543,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3">
-        <v>4500034381</v>
+        <v>4500037692</v>
       </c>
       <c r="B3">
         <v>10</v>
@@ -554,7 +554,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4">
-        <v>4500034382</v>
+        <v>4500037693</v>
       </c>
       <c r="B4">
         <v>10</v>
@@ -565,7 +565,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5">
-        <v>4500034376</v>
+        <v>4500037694</v>
       </c>
       <c r="B5">
         <v>10</v>
@@ -576,7 +576,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6">
-        <v>4500034377</v>
+        <v>4500037695</v>
       </c>
       <c r="B6">
         <v>10</v>
@@ -587,7 +587,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7">
-        <v>4500034378</v>
+        <v>4500037696</v>
       </c>
       <c r="B7">
         <v>10</v>
@@ -598,7 +598,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8">
-        <v>4500034379</v>
+        <v>4500037706</v>
       </c>
       <c r="B8">
         <v>10</v>
@@ -609,7 +609,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9">
-        <v>4500034380</v>
+        <v>4500037707</v>
       </c>
       <c r="B9">
         <v>10</v>
@@ -620,7 +620,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10">
-        <v>4500034365</v>
+        <v>4500037708</v>
       </c>
       <c r="B10">
         <v>10</v>
@@ -631,7 +631,7 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11">
-        <v>4500034366</v>
+        <v>4500037765</v>
       </c>
       <c r="B11">
         <v>10</v>
@@ -642,7 +642,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12">
-        <v>4500034367</v>
+        <v>4500037766</v>
       </c>
       <c r="B12">
         <v>10</v>
@@ -653,7 +653,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13">
-        <v>4500034368</v>
+        <v>4500037767</v>
       </c>
       <c r="B13">
         <v>10</v>
@@ -664,7 +664,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14">
-        <v>4500034369</v>
+        <v>4500037768</v>
       </c>
       <c r="B14">
         <v>10</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15">
-        <v>4500034370</v>
+        <v>4500037724</v>
       </c>
       <c r="B15">
         <v>10</v>
@@ -686,7 +686,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16">
-        <v>4500034371</v>
+        <v>4500037691</v>
       </c>
       <c r="B16">
         <v>10</v>
@@ -697,7 +697,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17">
-        <v>4500034372</v>
+        <v>4500037687</v>
       </c>
       <c r="B17">
         <v>10</v>
@@ -708,7 +708,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18">
-        <v>4500034373</v>
+        <v>4500037709</v>
       </c>
       <c r="B18">
         <v>10</v>
@@ -719,7 +719,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19">
-        <v>4500034374</v>
+        <v>4500037779</v>
       </c>
       <c r="B19">
         <v>10</v>
@@ -730,7 +730,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20">
-        <v>4500034375</v>
+        <v>4500037780</v>
       </c>
       <c r="B20">
         <v>10</v>
@@ -741,7 +741,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21">
-        <v>4500034355</v>
+        <v>4500037781</v>
       </c>
       <c r="B21">
         <v>10</v>
@@ -752,7 +752,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22">
-        <v>4500034356</v>
+        <v>4500037782</v>
       </c>
       <c r="B22">
         <v>10</v>
@@ -763,7 +763,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23">
-        <v>4500034357</v>
+        <v>4500037810</v>
       </c>
       <c r="B23">
         <v>10</v>
@@ -774,7 +774,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24">
-        <v>4500034358</v>
+        <v>4500037679</v>
       </c>
       <c r="B24">
         <v>10</v>
@@ -785,7 +785,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25">
-        <v>4500034359</v>
+        <v>4500037680</v>
       </c>
       <c r="B25">
         <v>10</v>
@@ -796,7 +796,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26">
-        <v>4500034360</v>
+        <v>4500037723</v>
       </c>
       <c r="B26">
         <v>10</v>
@@ -807,7 +807,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27">
-        <v>4500034361</v>
+        <v>4500037715</v>
       </c>
       <c r="B27">
         <v>10</v>
@@ -818,7 +818,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28">
-        <v>4500034362</v>
+        <v>4500037671</v>
       </c>
       <c r="B28">
         <v>10</v>
@@ -829,7 +829,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29">
-        <v>4500034293</v>
+        <v>4500037688</v>
       </c>
       <c r="B29">
         <v>10</v>
@@ -840,7 +840,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30">
-        <v>4500034294</v>
+        <v>4500037672</v>
       </c>
       <c r="B30">
         <v>10</v>
@@ -851,7 +851,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31">
-        <v>4500034295</v>
+        <v>4500037815</v>
       </c>
       <c r="B31">
         <v>10</v>
@@ -862,7 +862,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32">
-        <v>4500034296</v>
+        <v>4500037816</v>
       </c>
       <c r="B32">
         <v>10</v>
@@ -873,7 +873,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33">
-        <v>4500034297</v>
+        <v>4500037817</v>
       </c>
       <c r="B33">
         <v>10</v>
@@ -884,7 +884,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34">
-        <v>4500034298</v>
+        <v>4500037711</v>
       </c>
       <c r="B34">
         <v>10</v>
@@ -895,7 +895,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35">
-        <v>4500034299</v>
+        <v>4500037712</v>
       </c>
       <c r="B35">
         <v>10</v>
@@ -906,7 +906,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36">
-        <v>4500034300</v>
+        <v>4500037713</v>
       </c>
       <c r="B36">
         <v>10</v>
@@ -917,7 +917,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37">
-        <v>4500034301</v>
+        <v>4500037685</v>
       </c>
       <c r="B37">
         <v>10</v>
@@ -928,7 +928,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38">
-        <v>4500034302</v>
+        <v>4500037686</v>
       </c>
       <c r="B38">
         <v>10</v>
@@ -939,7 +939,7 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39">
-        <v>4500034303</v>
+        <v>4500037710</v>
       </c>
       <c r="B39">
         <v>10</v>
@@ -950,7 +950,7 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40">
-        <v>4500034304</v>
+        <v>4500037812</v>
       </c>
       <c r="B40">
         <v>10</v>
@@ -961,7 +961,7 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41">
-        <v>4500034305</v>
+        <v>4500037813</v>
       </c>
       <c r="B41">
         <v>10</v>
@@ -972,7 +972,7 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42">
-        <v>4500034306</v>
+        <v>4500037814</v>
       </c>
       <c r="B42">
         <v>10</v>
@@ -983,7 +983,7 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43">
-        <v>4500034307</v>
+        <v>4500037676</v>
       </c>
       <c r="B43">
         <v>10</v>
@@ -994,7 +994,7 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44">
-        <v>4500034308</v>
+        <v>4500037677</v>
       </c>
       <c r="B44">
         <v>10</v>
@@ -1005,7 +1005,7 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45">
-        <v>4500034309</v>
+        <v>4500037678</v>
       </c>
       <c r="B45">
         <v>10</v>
@@ -1016,7 +1016,7 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46">
-        <v>4500034310</v>
+        <v>4500037673</v>
       </c>
       <c r="B46">
         <v>10</v>
@@ -1027,7 +1027,7 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47">
-        <v>4500034315</v>
+        <v>4500037674</v>
       </c>
       <c r="B47">
         <v>10</v>
@@ -1038,7 +1038,7 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48">
-        <v>4500034316</v>
+        <v>4500037675</v>
       </c>
       <c r="B48">
         <v>10</v>
@@ -1049,7 +1049,7 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49">
-        <v>4500034317</v>
+        <v>4500037689</v>
       </c>
       <c r="B49">
         <v>10</v>
@@ -1060,7 +1060,7 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50">
-        <v>4500034318</v>
+        <v>4500037690</v>
       </c>
       <c r="B50">
         <v>10</v>
@@ -1071,7 +1071,7 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51">
-        <v>4500034319</v>
+        <v>4500037670</v>
       </c>
       <c r="B51">
         <v>10</v>
@@ -1082,7 +1082,7 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52">
-        <v>4500034320</v>
+        <v>4500037681</v>
       </c>
       <c r="B52">
         <v>10</v>
@@ -1093,7 +1093,7 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53">
-        <v>4500034321</v>
+        <v>4500037682</v>
       </c>
       <c r="B53">
         <v>10</v>
@@ -1104,7 +1104,7 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54">
-        <v>4500034322</v>
+        <v>4500037683</v>
       </c>
       <c r="B54">
         <v>10</v>
@@ -1115,7 +1115,7 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55">
-        <v>4500034323</v>
+        <v>4500037684</v>
       </c>
       <c r="B55">
         <v>10</v>
@@ -1126,7 +1126,7 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56">
-        <v>4500034324</v>
+        <v>4500037704</v>
       </c>
       <c r="B56">
         <v>10</v>
@@ -1137,7 +1137,7 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57">
-        <v>4500034325</v>
+        <v>4500037703</v>
       </c>
       <c r="B57">
         <v>10</v>
@@ -1148,7 +1148,7 @@
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58">
-        <v>4500034326</v>
+        <v>4500037702</v>
       </c>
       <c r="B58">
         <v>10</v>
@@ -1159,7 +1159,7 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59">
-        <v>4500034327</v>
+        <v>4500037701</v>
       </c>
       <c r="B59">
         <v>10</v>
@@ -1170,7 +1170,7 @@
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60">
-        <v>4500034328</v>
+        <v>4500037700</v>
       </c>
       <c r="B60">
         <v>10</v>
@@ -1181,7 +1181,7 @@
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61">
-        <v>4500034329</v>
+        <v>4500037699</v>
       </c>
       <c r="B61">
         <v>10</v>
@@ -1192,7 +1192,7 @@
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62">
-        <v>4500034330</v>
+        <v>4500037698</v>
       </c>
       <c r="B62">
         <v>10</v>
@@ -1203,7 +1203,7 @@
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63">
-        <v>4500034331</v>
+        <v>4500037697</v>
       </c>
       <c r="B63">
         <v>10</v>
@@ -1214,7 +1214,7 @@
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64">
-        <v>4500034332</v>
+        <v>4500037705</v>
       </c>
       <c r="B64">
         <v>10</v>
@@ -1225,7 +1225,7 @@
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65">
-        <v>4500034333</v>
+        <v>4500037714</v>
       </c>
       <c r="B65">
         <v>10</v>
@@ -1236,7 +1236,7 @@
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66">
-        <v>4500034334</v>
+        <v>4500037879</v>
       </c>
       <c r="B66">
         <v>10</v>
@@ -1247,7 +1247,7 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67">
-        <v>4500034335</v>
+        <v>4500037878</v>
       </c>
       <c r="B67">
         <v>10</v>
@@ -1258,7 +1258,7 @@
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68">
-        <v>4500034336</v>
+        <v>4500037877</v>
       </c>
       <c r="B68">
         <v>10</v>
@@ -1269,7 +1269,7 @@
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69">
-        <v>4500034337</v>
+        <v>4500037876</v>
       </c>
       <c r="B69">
         <v>10</v>
@@ -1280,7 +1280,7 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70">
-        <v>4500034338</v>
+        <v>4500037873</v>
       </c>
       <c r="B70">
         <v>10</v>
@@ -1291,7 +1291,7 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71">
-        <v>4500034339</v>
+        <v>4500037872</v>
       </c>
       <c r="B71">
         <v>10</v>
@@ -1302,7 +1302,7 @@
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72">
-        <v>4500034261</v>
+        <v>4500037871</v>
       </c>
       <c r="B72">
         <v>10</v>
@@ -1313,7 +1313,7 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73">
-        <v>4500034262</v>
+        <v>4500037870</v>
       </c>
       <c r="B73">
         <v>10</v>
@@ -1324,7 +1324,7 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74">
-        <v>4500034263</v>
+        <v>4500037869</v>
       </c>
       <c r="B74">
         <v>10</v>
@@ -1335,7 +1335,7 @@
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75">
-        <v>4500034264</v>
+        <v>4500037868</v>
       </c>
       <c r="B75">
         <v>10</v>
@@ -1346,7 +1346,7 @@
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76">
-        <v>4500034265</v>
+        <v>4500037867</v>
       </c>
       <c r="B76">
         <v>10</v>
@@ -1357,7 +1357,7 @@
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77">
-        <v>4500034432</v>
+        <v>4500037866</v>
       </c>
       <c r="B77">
         <v>10</v>
@@ -1368,7 +1368,7 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78">
-        <v>4500034431</v>
+        <v>4500037865</v>
       </c>
       <c r="B78">
         <v>10</v>
@@ -1379,7 +1379,7 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79">
-        <v>4500034435</v>
+        <v>4500037864</v>
       </c>
       <c r="B79">
         <v>10</v>
@@ -1390,7 +1390,7 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80">
-        <v>4500034434</v>
+        <v>4500037863</v>
       </c>
       <c r="B80">
         <v>10</v>
@@ -1401,7 +1401,7 @@
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81">
-        <v>4500034195</v>
+        <v>4500037862</v>
       </c>
       <c r="B81">
         <v>10</v>
@@ -1412,7 +1412,7 @@
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82">
-        <v>4500034197</v>
+        <v>4500037861</v>
       </c>
       <c r="B82">
         <v>10</v>
@@ -1423,7 +1423,7 @@
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83">
-        <v>4500034169</v>
+        <v>4500037874</v>
       </c>
       <c r="B83">
         <v>10</v>
@@ -1434,7 +1434,7 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84">
-        <v>4500034170</v>
+        <v>4500037875</v>
       </c>
       <c r="B84">
         <v>10</v>
@@ -1445,7 +1445,7 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85">
-        <v>4500034166</v>
+        <v>4500037860</v>
       </c>
       <c r="B85">
         <v>10</v>
@@ -1456,7 +1456,7 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86">
-        <v>4500034179</v>
+        <v>4500037859</v>
       </c>
       <c r="B86">
         <v>10</v>
@@ -1467,7 +1467,7 @@
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87">
-        <v>4500034167</v>
+        <v>4500037858</v>
       </c>
       <c r="B87">
         <v>10</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88">
-        <v>4500034209</v>
+        <v>4500037857</v>
       </c>
       <c r="B88">
         <v>10</v>
@@ -1489,7 +1489,7 @@
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89">
-        <v>4500034178</v>
+        <v>4500037856</v>
       </c>
       <c r="B89">
         <v>10</v>
@@ -1500,7 +1500,7 @@
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90">
-        <v>4500034171</v>
+        <v>4500037851</v>
       </c>
       <c r="B90">
         <v>10</v>
@@ -1511,7 +1511,7 @@
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91">
-        <v>4500034174</v>
+        <v>4500037852</v>
       </c>
       <c r="B91">
         <v>10</v>
@@ -1522,7 +1522,7 @@
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92">
-        <v>4500034187</v>
+        <v>4500037853</v>
       </c>
       <c r="B92">
         <v>10</v>
@@ -1533,7 +1533,7 @@
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A93">
-        <v>4500034165</v>
+        <v>4500037854</v>
       </c>
       <c r="B93">
         <v>10</v>
@@ -1544,7 +1544,7 @@
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A94">
-        <v>4500034172</v>
+        <v>4500037855</v>
       </c>
       <c r="B94">
         <v>10</v>
@@ -1555,7 +1555,7 @@
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A95">
-        <v>4500034182</v>
+        <v>4500037850</v>
       </c>
       <c r="B95">
         <v>10</v>
@@ -1566,7 +1566,7 @@
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96">
-        <v>4500034185</v>
+        <v>4500037849</v>
       </c>
       <c r="B96">
         <v>10</v>
@@ -1577,7 +1577,7 @@
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97">
-        <v>4500034184</v>
+        <v>4500037848</v>
       </c>
       <c r="B97">
         <v>10</v>
@@ -1588,7 +1588,7 @@
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A98">
-        <v>4500034191</v>
+        <v>4500037847</v>
       </c>
       <c r="B98">
         <v>10</v>
@@ -1599,7 +1599,7 @@
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A99">
-        <v>4500034211</v>
+        <v>4500037846</v>
       </c>
       <c r="B99">
         <v>10</v>
@@ -1610,7 +1610,7 @@
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A100">
-        <v>4500034176</v>
+        <v>4500037845</v>
       </c>
       <c r="B100">
         <v>10</v>
@@ -1621,7 +1621,7 @@
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101">
-        <v>4500034230</v>
+        <v>4500037844</v>
       </c>
       <c r="B101">
         <v>10</v>
@@ -1632,7 +1632,7 @@
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A102">
-        <v>4500034190</v>
+        <v>4500037843</v>
       </c>
       <c r="B102">
         <v>10</v>
@@ -1643,7 +1643,7 @@
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A103">
-        <v>4500034181</v>
+        <v>4500037842</v>
       </c>
       <c r="B103">
         <v>10</v>
@@ -1654,7 +1654,7 @@
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A104">
-        <v>4500034183</v>
+        <v>4500037841</v>
       </c>
       <c r="B104">
         <v>10</v>
@@ -1665,7 +1665,7 @@
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A105">
-        <v>4500034189</v>
+        <v>4500037840</v>
       </c>
       <c r="B105">
         <v>10</v>
@@ -1676,7 +1676,7 @@
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106">
-        <v>4500034192</v>
+        <v>4500037839</v>
       </c>
       <c r="B106">
         <v>10</v>
@@ -1687,7 +1687,7 @@
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107">
-        <v>4500034168</v>
+        <v>4500037838</v>
       </c>
       <c r="B107">
         <v>10</v>
@@ -1698,7 +1698,7 @@
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A108">
-        <v>4500034180</v>
+        <v>4500037837</v>
       </c>
       <c r="B108">
         <v>10</v>
@@ -1709,7 +1709,7 @@
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A109">
-        <v>4500034175</v>
+        <v>4500037834</v>
       </c>
       <c r="B109">
         <v>10</v>
@@ -1720,7 +1720,7 @@
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A110">
-        <v>4500034173</v>
+        <v>4500037835</v>
       </c>
       <c r="B110">
         <v>10</v>
@@ -1731,7 +1731,7 @@
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A111">
-        <v>4500034208</v>
+        <v>4500037836</v>
       </c>
       <c r="B111">
         <v>10</v>
@@ -1742,7 +1742,7 @@
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A112">
-        <v>4500034188</v>
+        <v>4500037833</v>
       </c>
       <c r="B112">
         <v>10</v>
@@ -1753,7 +1753,7 @@
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113">
-        <v>4500034186</v>
+        <v>4500037883</v>
       </c>
       <c r="B113">
         <v>10</v>
@@ -1764,7 +1764,7 @@
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114">
-        <v>4500034203</v>
+        <v>4500037884</v>
       </c>
       <c r="B114">
         <v>10</v>
@@ -1775,7 +1775,7 @@
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115">
-        <v>4500034433</v>
+        <v>4500037808</v>
       </c>
       <c r="B115">
         <v>10</v>
@@ -1786,7 +1786,7 @@
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116">
-        <v>4500034177</v>
+        <v>4500037807</v>
       </c>
       <c r="B116">
         <v>10</v>
@@ -1797,7 +1797,7 @@
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117">
-        <v>4500034287</v>
+        <v>4500037806</v>
       </c>
       <c r="B117">
         <v>10</v>
@@ -1808,7 +1808,7 @@
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118">
-        <v>4500034349</v>
+        <v>4500037801</v>
       </c>
       <c r="B118">
         <v>10</v>
@@ -1819,7 +1819,7 @@
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119">
-        <v>4500034350</v>
+        <v>4500037802</v>
       </c>
       <c r="B119">
         <v>10</v>
@@ -1830,7 +1830,7 @@
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120">
-        <v>4500034386</v>
+        <v>4500037803</v>
       </c>
       <c r="B120">
         <v>10</v>
@@ -1841,7 +1841,7 @@
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121">
-        <v>4500034241</v>
+        <v>4500037804</v>
       </c>
       <c r="B121">
         <v>10</v>
@@ -1852,7 +1852,7 @@
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122">
-        <v>4500034342</v>
+        <v>4500037805</v>
       </c>
       <c r="B122">
         <v>10</v>
@@ -1863,7 +1863,7 @@
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123">
-        <v>4500034343</v>
+        <v>4500037800</v>
       </c>
       <c r="B123">
         <v>10</v>
@@ -1874,7 +1874,7 @@
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124">
-        <v>4500034344</v>
+        <v>4500037799</v>
       </c>
       <c r="B124">
         <v>10</v>
@@ -1885,7 +1885,7 @@
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125">
-        <v>4500034259</v>
+        <v>4500037797</v>
       </c>
       <c r="B125">
         <v>10</v>
@@ -1896,7 +1896,7 @@
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126">
-        <v>4500034260</v>
+        <v>4500037798</v>
       </c>
       <c r="B126">
         <v>10</v>
@@ -1907,7 +1907,7 @@
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127">
-        <v>4500034266</v>
+        <v>4500037796</v>
       </c>
       <c r="B127">
         <v>10</v>
@@ -1918,7 +1918,7 @@
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128">
-        <v>4500034257</v>
+        <v>4500037795</v>
       </c>
       <c r="B128">
         <v>10</v>
@@ -1929,7 +1929,7 @@
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129">
-        <v>4500034258</v>
+        <v>4500037794</v>
       </c>
       <c r="B129">
         <v>10</v>
@@ -1940,7 +1940,7 @@
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A130">
-        <v>4500034270</v>
+        <v>4500037793</v>
       </c>
       <c r="B130">
         <v>10</v>
@@ -1951,7 +1951,7 @@
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131">
-        <v>4500034271</v>
+        <v>4500037792</v>
       </c>
       <c r="B131">
         <v>10</v>
@@ -1962,7 +1962,7 @@
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132">
-        <v>4500034272</v>
+        <v>4500037791</v>
       </c>
       <c r="B132">
         <v>10</v>
@@ -1973,7 +1973,7 @@
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133">
-        <v>4500034267</v>
+        <v>4500037790</v>
       </c>
       <c r="B133">
         <v>10</v>
@@ -1984,7 +1984,7 @@
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134">
-        <v>4500034268</v>
+        <v>4500037789</v>
       </c>
       <c r="B134">
         <v>10</v>
@@ -1995,7 +1995,7 @@
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135">
-        <v>4500034269</v>
+        <v>4500037788</v>
       </c>
       <c r="B135">
         <v>10</v>
@@ -2006,7 +2006,7 @@
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136">
-        <v>4500034273</v>
+        <v>4500037787</v>
       </c>
       <c r="B136">
         <v>10</v>
@@ -2017,7 +2017,7 @@
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A137">
-        <v>4500034274</v>
+        <v>4500037786</v>
       </c>
       <c r="B137">
         <v>10</v>
@@ -2028,7 +2028,7 @@
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A138">
-        <v>4500034346</v>
+        <v>4500037785</v>
       </c>
       <c r="B138">
         <v>10</v>
@@ -2039,7 +2039,7 @@
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A139">
-        <v>4500034275</v>
+        <v>4500037784</v>
       </c>
       <c r="B139">
         <v>10</v>
@@ -2050,7 +2050,7 @@
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A140">
-        <v>4500034391</v>
+        <v>4500037783</v>
       </c>
       <c r="B140">
         <v>10</v>
@@ -2061,7 +2061,7 @@
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A141">
-        <v>4500034403</v>
+        <v>4500037778</v>
       </c>
       <c r="B141">
         <v>10</v>
@@ -2072,7 +2072,7 @@
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A142">
-        <v>4500034404</v>
+        <v>4500037777</v>
       </c>
       <c r="B142">
         <v>10</v>
@@ -2083,7 +2083,7 @@
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A143">
-        <v>4500034405</v>
+        <v>4500037776</v>
       </c>
       <c r="B143">
         <v>10</v>
@@ -2094,7 +2094,7 @@
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A144">
-        <v>4500034406</v>
+        <v>4500037775</v>
       </c>
       <c r="B144">
         <v>10</v>
@@ -2105,7 +2105,7 @@
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145">
-        <v>4500034407</v>
+        <v>4500037774</v>
       </c>
       <c r="B145">
         <v>10</v>
@@ -2116,7 +2116,7 @@
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146">
-        <v>4500034408</v>
+        <v>4500037773</v>
       </c>
       <c r="B146">
         <v>10</v>
@@ -2127,7 +2127,7 @@
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147">
-        <v>4500034409</v>
+        <v>4500037772</v>
       </c>
       <c r="B147">
         <v>10</v>
@@ -2138,7 +2138,7 @@
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A148">
-        <v>4500034401</v>
+        <v>4500037771</v>
       </c>
       <c r="B148">
         <v>10</v>
@@ -2149,7 +2149,7 @@
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149">
-        <v>4500034421</v>
+        <v>4500037770</v>
       </c>
       <c r="B149">
         <v>10</v>
@@ -2160,7 +2160,7 @@
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150">
-        <v>4500034390</v>
+        <v>4500037825</v>
       </c>
       <c r="B150">
         <v>10</v>
@@ -2171,7 +2171,7 @@
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151">
-        <v>4500034392</v>
+        <v>4500037824</v>
       </c>
       <c r="B151">
         <v>10</v>
@@ -2182,7 +2182,7 @@
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152">
-        <v>4500034393</v>
+        <v>4500037823</v>
       </c>
       <c r="B152">
         <v>10</v>
@@ -2193,7 +2193,7 @@
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A153">
-        <v>4500034394</v>
+        <v>4500037822</v>
       </c>
       <c r="B153">
         <v>10</v>
@@ -2204,7 +2204,7 @@
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A154">
-        <v>4500034395</v>
+        <v>4500037821</v>
       </c>
       <c r="B154">
         <v>10</v>
@@ -2215,7 +2215,7 @@
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A155">
-        <v>4500034412</v>
+        <v>4500037820</v>
       </c>
       <c r="B155">
         <v>10</v>
@@ -2226,7 +2226,7 @@
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A156">
-        <v>4500034430</v>
+        <v>4500037819</v>
       </c>
       <c r="B156">
         <v>10</v>
@@ -2237,7 +2237,7 @@
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A157">
-        <v>4500034397</v>
+        <v>4500037818</v>
       </c>
       <c r="B157">
         <v>10</v>
@@ -2248,7 +2248,7 @@
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A158">
-        <v>4500034398</v>
+        <v>4500037831</v>
       </c>
       <c r="B158">
         <v>10</v>
@@ -2259,7 +2259,7 @@
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A159">
-        <v>4500034399</v>
+        <v>4500037830</v>
       </c>
       <c r="B159">
         <v>10</v>
@@ -2270,7 +2270,7 @@
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160">
-        <v>4500034396</v>
+        <v>4500037829</v>
       </c>
       <c r="B160">
         <v>10</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161">
-        <v>4500034400</v>
+        <v>4500037828</v>
       </c>
       <c r="B161">
         <v>10</v>
@@ -2292,7 +2292,7 @@
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162">
-        <v>4500034422</v>
+        <v>4500037827</v>
       </c>
       <c r="B162">
         <v>10</v>
@@ -2303,7 +2303,7 @@
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163">
-        <v>4500034410</v>
+        <v>4500037826</v>
       </c>
       <c r="B163">
         <v>10</v>
@@ -2314,7 +2314,7 @@
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A164">
-        <v>4500034387</v>
+        <v>4500037764</v>
       </c>
       <c r="B164">
         <v>10</v>
@@ -2325,7 +2325,7 @@
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A165">
-        <v>4500034388</v>
+        <v>4500037763</v>
       </c>
       <c r="B165">
         <v>10</v>
@@ -2336,7 +2336,7 @@
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A166">
-        <v>4500034389</v>
+        <v>4500037762</v>
       </c>
       <c r="B166">
         <v>10</v>
@@ -2347,7 +2347,7 @@
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A167">
-        <v>4500034427</v>
+        <v>4500037761</v>
       </c>
       <c r="B167">
         <v>10</v>
@@ -2358,7 +2358,7 @@
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A168">
-        <v>4500034413</v>
+        <v>4500037756</v>
       </c>
       <c r="B168">
         <v>10</v>
@@ -2369,7 +2369,7 @@
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A169">
-        <v>4500034402</v>
+        <v>4500037757</v>
       </c>
       <c r="B169">
         <v>10</v>
@@ -2380,7 +2380,7 @@
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A170">
-        <v>4500034415</v>
+        <v>4500037758</v>
       </c>
       <c r="B170">
         <v>10</v>
@@ -2391,7 +2391,7 @@
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A171">
-        <v>4500034417</v>
+        <v>4500037759</v>
       </c>
       <c r="B171">
         <v>10</v>
@@ -2402,7 +2402,7 @@
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A172">
-        <v>4500034414</v>
+        <v>4500037760</v>
       </c>
       <c r="B172">
         <v>10</v>
@@ -2413,7 +2413,7 @@
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A173">
-        <v>4500034411</v>
+        <v>4500037755</v>
       </c>
       <c r="B173">
         <v>10</v>
@@ -2424,7 +2424,7 @@
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A174">
-        <v>4500034416</v>
+        <v>4500037754</v>
       </c>
       <c r="B174">
         <v>10</v>
@@ -2435,7 +2435,7 @@
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A175">
-        <v>4500034429</v>
+        <v>4500037753</v>
       </c>
       <c r="B175">
         <v>10</v>
@@ -2446,7 +2446,7 @@
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A176">
-        <v>4500034428</v>
+        <v>4500037748</v>
       </c>
       <c r="B176">
         <v>10</v>
@@ -2457,7 +2457,7 @@
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A177">
-        <v>4500034420</v>
+        <v>4500037749</v>
       </c>
       <c r="B177">
         <v>10</v>
@@ -2468,7 +2468,7 @@
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A178">
-        <v>4500034423</v>
+        <v>4500037750</v>
       </c>
       <c r="B178">
         <v>10</v>
@@ -2479,7 +2479,7 @@
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A179">
-        <v>4500034418</v>
+        <v>4500037751</v>
       </c>
       <c r="B179">
         <v>10</v>
@@ -2490,7 +2490,7 @@
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A180">
-        <v>4500034419</v>
+        <v>4500037752</v>
       </c>
       <c r="B180">
         <v>10</v>
@@ -2501,7 +2501,7 @@
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A181">
-        <v>4500034424</v>
+        <v>4500037747</v>
       </c>
       <c r="B181">
         <v>10</v>
@@ -2512,7 +2512,7 @@
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A182">
-        <v>4500034425</v>
+        <v>4500037746</v>
       </c>
       <c r="B182">
         <v>10</v>
@@ -2523,12 +2523,221 @@
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A183">
-        <v>4500034426</v>
+        <v>4500037745</v>
       </c>
       <c r="B183">
         <v>10</v>
       </c>
       <c r="E183" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A184">
+        <v>4500037744</v>
+      </c>
+      <c r="B184">
+        <v>10</v>
+      </c>
+      <c r="E184" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A185">
+        <v>4500037743</v>
+      </c>
+      <c r="B185">
+        <v>10</v>
+      </c>
+      <c r="E185" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A186">
+        <v>4500037738</v>
+      </c>
+      <c r="B186">
+        <v>10</v>
+      </c>
+      <c r="E186" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A187">
+        <v>4500037739</v>
+      </c>
+      <c r="B187">
+        <v>10</v>
+      </c>
+      <c r="E187" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A188">
+        <v>4500037740</v>
+      </c>
+      <c r="B188">
+        <v>10</v>
+      </c>
+      <c r="E188" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A189">
+        <v>4500037741</v>
+      </c>
+      <c r="B189">
+        <v>10</v>
+      </c>
+      <c r="E189" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A190">
+        <v>4500037742</v>
+      </c>
+      <c r="B190">
+        <v>10</v>
+      </c>
+      <c r="E190" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A191">
+        <v>4500037737</v>
+      </c>
+      <c r="B191">
+        <v>10</v>
+      </c>
+      <c r="E191" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A192">
+        <v>4500037736</v>
+      </c>
+      <c r="B192">
+        <v>10</v>
+      </c>
+      <c r="E192" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A193">
+        <v>4500037735</v>
+      </c>
+      <c r="B193">
+        <v>10</v>
+      </c>
+      <c r="E193" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A194">
+        <v>4500037734</v>
+      </c>
+      <c r="B194">
+        <v>10</v>
+      </c>
+      <c r="E194" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A195">
+        <v>4500037733</v>
+      </c>
+      <c r="B195">
+        <v>10</v>
+      </c>
+      <c r="E195" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A196">
+        <v>4500037732</v>
+      </c>
+      <c r="B196">
+        <v>10</v>
+      </c>
+      <c r="E196" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A197">
+        <v>4500037731</v>
+      </c>
+      <c r="B197">
+        <v>10</v>
+      </c>
+      <c r="E197" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A198">
+        <v>4500037730</v>
+      </c>
+      <c r="B198">
+        <v>10</v>
+      </c>
+      <c r="E198" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A199">
+        <v>4500037729</v>
+      </c>
+      <c r="B199">
+        <v>10</v>
+      </c>
+      <c r="E199" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A200">
+        <v>4500037728</v>
+      </c>
+      <c r="B200">
+        <v>10</v>
+      </c>
+      <c r="E200" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A201">
+        <v>4500037727</v>
+      </c>
+      <c r="B201">
+        <v>10</v>
+      </c>
+      <c r="E201" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A202">
+        <v>4500037726</v>
+      </c>
+      <c r="B202">
+        <v>10</v>
+      </c>
+      <c r="E202" s="1" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>